<commit_message>
adding iucn categories and re-running
</commit_message>
<xml_diff>
--- a/data/hypothesis_names.xlsx
+++ b/data/hypothesis_names.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Amelia DuVall\Dropbox\UW-SAFS\Research\CHIS_CVoI_seabirds\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajduvall/Dropbox/UW-SAFS/Manuscripts/DuVall_etal_CVOI/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E449F3-9C5D-4B5A-8101-B89878C1C5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A93D7A78-C3A1-8346-8907-1D4B1CC48B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14483" yWindow="0" windowWidth="14566" windowHeight="15563" xr2:uid="{34BF7D82-81FA-4454-B10C-E67DAFCD4B4B}"/>
+    <workbookView xWindow="-30440" yWindow="900" windowWidth="25540" windowHeight="15960" xr2:uid="{34BF7D82-81FA-4454-B10C-E67DAFCD4B4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -237,13 +237,34 @@
   </si>
   <si>
     <t>Toxins/diseases/parasites</t>
+  </si>
+  <si>
+    <t>IUCN_Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy production &amp; mining </t>
+  </si>
+  <si>
+    <t>Transportation &amp; service corridors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biological resource use </t>
+  </si>
+  <si>
+    <t>Human intrusions &amp; disturbance</t>
+  </si>
+  <si>
+    <t>Invasive &amp; other problematic species, genes &amp; diseases</t>
+  </si>
+  <si>
+    <t>Climate change &amp; severe weather</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,6 +277,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="2">
@@ -278,8 +304,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,13 +641,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FB65730-CDB0-41B3-8694-0FFD2C965F97}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -630,8 +658,11 @@
       <c r="C1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -641,8 +672,11 @@
       <c r="C2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -652,8 +686,11 @@
       <c r="C3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -663,8 +700,11 @@
       <c r="C4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -674,8 +714,11 @@
       <c r="C5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -685,8 +728,11 @@
       <c r="C6" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -696,8 +742,11 @@
       <c r="C7" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -707,8 +756,11 @@
       <c r="C8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -718,8 +770,11 @@
       <c r="C9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -729,8 +784,11 @@
       <c r="C10" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -740,8 +798,11 @@
       <c r="C11" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>62</v>
       </c>
@@ -751,8 +812,11 @@
       <c r="C12" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -762,8 +826,11 @@
       <c r="C13" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>63</v>
       </c>
@@ -773,8 +840,11 @@
       <c r="C14" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>63</v>
       </c>
@@ -784,8 +854,11 @@
       <c r="C15" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>64</v>
       </c>
@@ -795,8 +868,11 @@
       <c r="C16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -806,8 +882,11 @@
       <c r="C17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>64</v>
       </c>
@@ -817,8 +896,11 @@
       <c r="C18" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -828,8 +910,11 @@
       <c r="C19" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>65</v>
       </c>
@@ -839,8 +924,11 @@
       <c r="C20" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -850,8 +938,11 @@
       <c r="C21" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -861,8 +952,11 @@
       <c r="C22" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -872,8 +966,11 @@
       <c r="C23" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D23" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -883,8 +980,11 @@
       <c r="C24" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D24" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -894,8 +994,11 @@
       <c r="C25" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D25" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>65</v>
       </c>
@@ -905,8 +1008,11 @@
       <c r="C26" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D26" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>66</v>
       </c>
@@ -916,8 +1022,11 @@
       <c r="C27" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D27" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>66</v>
       </c>
@@ -927,8 +1036,11 @@
       <c r="C28" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>66</v>
       </c>
@@ -937,6 +1049,9 @@
       </c>
       <c r="C29" t="s">
         <v>57</v>
+      </c>
+      <c r="D29" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>